<commit_message>
fix import issue in server
</commit_message>
<xml_diff>
--- a/excel_files/DPR.xlsx
+++ b/excel_files/DPR.xlsx
@@ -11422,10 +11422,8 @@
       <c r="BT30" s="59" t="n">
         <v>53.65</v>
       </c>
-      <c r="BU30" s="59" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="BU30" s="59" t="n">
+        <v>25</v>
       </c>
       <c r="BV30" s="59" t="n">
         <v>53.65</v>
@@ -31880,7 +31878,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32025,43 +32023,87 @@
     </row>
     <row r="4">
       <c r="A4" s="71" t="n">
-        <v>45858.87873857176</v>
-      </c>
-      <c r="B4" t="inlineStr">
+        <v>45858.87873857639</v>
+      </c>
+      <c r="B4" s="32" t="inlineStr">
         <is>
           <t>July.25</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="32" t="inlineStr">
         <is>
           <t>ashish</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="32" t="inlineStr">
         <is>
           <t>baraiy</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="32" t="inlineStr">
         <is>
           <t>25 kg of structural steel has be done</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="32" t="inlineStr">
         <is>
           <t>Structural Steel</t>
         </is>
       </c>
-      <c r="G4" t="n">
+      <c r="G4" s="32" t="n">
         <v>30</v>
       </c>
-      <c r="H4" t="n">
+      <c r="H4" s="32" t="n">
         <v>71</v>
       </c>
-      <c r="I4" t="n">
+      <c r="I4" s="32" t="n">
         <v>25</v>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J4" s="32" t="inlineStr">
+        <is>
+          <t>Structural Steel is updated with 25.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="71" t="n">
+        <v>45859.61774286338</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>July.25</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ashish</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>baraiya</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>25 kg of structural steel has been updated</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>30</v>
+      </c>
+      <c r="H5" t="n">
+        <v>73</v>
+      </c>
+      <c r="I5" t="n">
+        <v>25</v>
+      </c>
+      <c r="J5" t="inlineStr">
         <is>
           <t>Structural Steel is updated with 25.0</t>
         </is>

</xml_diff>